<commit_message>
add ref to RNIV c54165e80da950ff43816ad7b38aca27fb88924a
</commit_message>
<xml_diff>
--- a/ig/nr-add-def-ins-collection/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-add-def-ins-collection/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-06T10:34:42+00:00</t>
+    <t>2023-11-06T13:10:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil FrPatient appliqué à l'INS avec identité validée.</t>
+    <t>Profil FrPatient appliqué à l'INS avec identité validée. Pour plus d'informations, consulter le référentiel national d'identitovigilance de l'ANS (RNIV).</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
add ref to INS doc a7277c4a487e8d0703ddde8a992d70f82f920a4b
</commit_message>
<xml_diff>
--- a/ig/nr-add-def-ins-collection/StructureDefinition-fr-core-patient-ins.xlsx
+++ b/ig/nr-add-def-ins-collection/StructureDefinition-fr-core-patient-ins.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-11-06T13:10:33+00:00</t>
+    <t>2023-11-06T13:11:32+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Profil FrPatient appliqué à l'INS avec identité validée. Pour plus d'informations, consulter le référentiel national d'identitovigilance de l'ANS (RNIV).</t>
+    <t>Profil FrPatient appliqué à l'INS avec identité validée. Pour plus d'informations sur le contexte du patient INS, consultez le référentiel national d'identitovigilance (RNIV) et la documentation du référentiel INS de l'ANS .</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>